<commit_message>
fix: remove lark2json file & update translations.xlsx
</commit_message>
<xml_diff>
--- a/scripts/xlsx2json/translations.xlsx
+++ b/scripts/xlsx2json/translations.xlsx
@@ -227,7 +227,7 @@
     <t>message.error_1203</t>
   </si>
   <si>
-    <t>您上一次的提款被拒絕。請等待 {{time}} 分鐘後再嘗試。</t>
+    <t>您上一次的提款被拒绝。请等待 {{time}} 分钟后再尝试。</t>
   </si>
   <si>
     <t>Your last withdrawal was decllined. Please wait {{time}} minutes before trying again.</t>
@@ -859,7 +859,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -869,19 +869,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1470,7 +1458,7 @@
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" ht="17" spans="1:6">
       <c r="A3" s="2" t="s">
@@ -1584,7 +1572,7 @@
       <c r="A9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -1602,16 +1590,16 @@
       <c r="A10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="3" t="s">
         <v>49</v>
       </c>
       <c r="F10" s="2"/>
@@ -1620,16 +1608,16 @@
       <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="3" t="s">
         <v>54</v>
       </c>
       <c r="F11" s="2"/>
@@ -1638,16 +1626,16 @@
       <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="3" t="s">
         <v>59</v>
       </c>
       <c r="F12" s="2"/>
@@ -1656,16 +1644,16 @@
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="3" t="s">
         <v>64</v>
       </c>
       <c r="F13" s="2"/>
@@ -1677,28 +1665,28 @@
       <c r="B14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="4" t="s">
         <v>69</v>
       </c>
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="B15" s="5"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="B16" s="5"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: update xlsx2json script
</commit_message>
<xml_diff>
--- a/scripts/xlsx2json/translations.xlsx
+++ b/scripts/xlsx2json/translations.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="72">
   <si>
     <t>key</t>
   </si>
@@ -237,6 +237,12 @@
   </si>
   <si>
     <t>Tu último retiro fue rechazado. Por favor espera {{time}} minutos antes de intentarlo de nuevo.</t>
+  </si>
+  <si>
+    <t>message.error_1204</t>
+  </si>
+  <si>
+    <t>余额不足，请充值。</t>
   </si>
 </sst>
 </file>
@@ -1676,8 +1682,13 @@
       </c>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:6">
-      <c r="B15" s="3"/>
+    <row r="15" ht="17" spans="1:6">
+      <c r="A15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>

</xml_diff>